<commit_message>
feat: add Jalal Sons scraper (5th store), tune matching (681 groups, 7014 rows), update dashboard
</commit_message>
<xml_diff>
--- a/analysis/results/category_dispersion.xlsx
+++ b/analysis/results/category_dispersion.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,26 +425,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>avg_cv</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>avg_range</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>num_products</t>
         </is>
@@ -441,14 +453,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jellies and Marshmallows</t>
+          <t>chocolates</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85.71666666666665</v>
+        <v>71.15666666666665</v>
       </c>
       <c r="C2" t="n">
-        <v>541.6666666666666</v>
+        <v>679.6666666666666</v>
       </c>
       <c r="D2" t="n">
         <v>3</v>
@@ -457,30 +469,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fresh Vegetables</t>
+          <t>Tea</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>74.09833333333334</v>
+        <v>66.94800000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>243.3333333333333</v>
+        <v>1074.8</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>flour-atta</t>
+          <t>Sponges</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60.13</v>
+        <v>61.43</v>
       </c>
       <c r="C4" t="n">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -489,94 +501,94 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>chocolates</t>
+          <t>Canned Fruits</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>59.185</v>
+        <v>58.58</v>
       </c>
       <c r="C5" t="n">
-        <v>237.5</v>
+        <v>2301</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nutritional Drinks</t>
+          <t>meat-poultry</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50.86</v>
+        <v>57.12</v>
       </c>
       <c r="C6" t="n">
-        <v>835</v>
+        <v>3113.090909090909</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Chicken</t>
+          <t>Flavored Milk</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>49.5275</v>
+        <v>55.72</v>
       </c>
       <c r="C7" t="n">
-        <v>434</v>
+        <v>277</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cakes and Chocolates</t>
+          <t>pet-care</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>48.54882352941177</v>
+        <v>52.56</v>
       </c>
       <c r="C8" t="n">
-        <v>873.5882352941177</v>
+        <v>3338.076923076923</v>
       </c>
       <c r="D8" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Coffee and Whiteners</t>
+          <t>cooking-oil-ghee</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>46.09875</v>
+        <v>49.054</v>
       </c>
       <c r="C9" t="n">
-        <v>1155.5</v>
+        <v>4365</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Buns</t>
+          <t>Coffee and Whiteners</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>45.38</v>
+        <v>46.47</v>
       </c>
       <c r="C10" t="n">
-        <v>59</v>
+        <v>2005</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -585,318 +597,318 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Toilet Supplies</t>
+          <t>beverages</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44.99222222222222</v>
+        <v>45.53599999999999</v>
       </c>
       <c r="C11" t="n">
-        <v>568.1111111111111</v>
+        <v>1319.933333333333</v>
       </c>
       <c r="D11" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dishwashing Bars</t>
+          <t>snacks-beverages</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>39.41</v>
+        <v>43.12111111111111</v>
       </c>
       <c r="C12" t="n">
-        <v>73.33333333333333</v>
+        <v>388.7777777777778</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Flavored Milk</t>
+          <t>Toilet Supplies</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>38.634</v>
+        <v>42.51333333333334</v>
       </c>
       <c r="C13" t="n">
-        <v>459.0666666666667</v>
+        <v>730.6666666666666</v>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Detergents and Laundry Soaps</t>
+          <t>breakfast</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>38.05666666666666</v>
+        <v>41.93</v>
       </c>
       <c r="C14" t="n">
-        <v>347.9166666666667</v>
+        <v>2205</v>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>dairy</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35.3584</v>
+        <v>39.51846153846154</v>
       </c>
       <c r="C15" t="n">
-        <v>1910.76</v>
+        <v>1123.615384615385</v>
       </c>
       <c r="D15" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Canned Fruits</t>
+          <t>flour-atta</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>34.27333333333333</v>
+        <v>39.09</v>
       </c>
       <c r="C16" t="n">
-        <v>1051.333333333333</v>
+        <v>149.5</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tea</t>
+          <t>dairy-bakery</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31.97833333333334</v>
+        <v>35.27</v>
       </c>
       <c r="C17" t="n">
-        <v>570.1944444444445</v>
+        <v>200</v>
       </c>
       <c r="D17" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Products</t>
+          <t>Cakes and Chocolates</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>30.81866666666667</v>
+        <v>33.70666666666667</v>
       </c>
       <c r="C18" t="n">
-        <v>1027.1635</v>
+        <v>79.66666666666667</v>
       </c>
       <c r="D18" t="n">
-        <v>60</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sponges</t>
+          <t>household</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>30.14818181818182</v>
+        <v>33.24</v>
       </c>
       <c r="C19" t="n">
-        <v>483.3636363636364</v>
+        <v>354.6666666666667</v>
       </c>
       <c r="D19" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>dairy</t>
+          <t>personal-care</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>29.83555555555555</v>
+        <v>30.828</v>
       </c>
       <c r="C20" t="n">
-        <v>388</v>
+        <v>534.6</v>
       </c>
       <c r="D20" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>staples</t>
+          <t>Red Syrups</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>28.86444444444444</v>
+        <v>30.18</v>
       </c>
       <c r="C21" t="n">
-        <v>304.6666666666667</v>
+        <v>659</v>
       </c>
       <c r="D21" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Squashes</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>28.436</v>
+        <v>28.86702508960573</v>
       </c>
       <c r="C22" t="n">
-        <v>191</v>
+        <v>978.9995698924731</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>279</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Air Sprays</t>
+          <t>fruits-vegetables</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>28.102</v>
+        <v>28.715</v>
       </c>
       <c r="C23" t="n">
-        <v>167.6</v>
+        <v>615</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Disinfectants</t>
+          <t>Detergents and Laundry Soaps</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>27.9</v>
+        <v>27.5125</v>
       </c>
       <c r="C24" t="n">
-        <v>742.6</v>
+        <v>188.25</v>
       </c>
       <c r="D24" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>personal-care</t>
+          <t>Jams, Honey and Spreads</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>26.61</v>
+        <v>26.71</v>
       </c>
       <c r="C25" t="n">
-        <v>496.2</v>
+        <v>1499</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cheese</t>
+          <t>Insecticides</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>26.04923076923077</v>
+        <v>25.97666666666667</v>
       </c>
       <c r="C26" t="n">
-        <v>859</v>
+        <v>472.3333333333333</v>
       </c>
       <c r="D26" t="n">
-        <v>39</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dry Fruits and Nuts</t>
+          <t>tea-coffee</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>25.26</v>
+        <v>25.4</v>
       </c>
       <c r="C27" t="n">
-        <v>925.6</v>
+        <v>1208.416666666667</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Oils and Serums</t>
+          <t>Jellies and Custards</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>25.12</v>
+        <v>23.6425</v>
       </c>
       <c r="C28" t="n">
-        <v>541.3333333333334</v>
+        <v>66</v>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Sweets and Toffees</t>
+          <t>snacks</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>22.404</v>
+        <v>22.47307692307692</v>
       </c>
       <c r="C29" t="n">
-        <v>64.40000000000001</v>
+        <v>100.4615384615385</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pulses</t>
+          <t>Noodles and Pasta</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>21.808</v>
+        <v>22.194</v>
       </c>
       <c r="C30" t="n">
-        <v>167</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="D30" t="n">
         <v>5</v>
@@ -905,305 +917,305 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>fruits-vegetables</t>
+          <t>general</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>21.39</v>
+        <v>21.99582524271845</v>
       </c>
       <c r="C31" t="n">
-        <v>230</v>
+        <v>541.8955339805825</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>206</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Noodles and Pasta</t>
+          <t>Kebab and Koftas</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>21.14590909090909</v>
+        <v>19.815</v>
       </c>
       <c r="C32" t="n">
-        <v>108.4545454545455</v>
+        <v>406.5</v>
       </c>
       <c r="D32" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Dishwashing Liquids</t>
+          <t>Baby Milk</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>20.88625</v>
+        <v>19.13</v>
       </c>
       <c r="C33" t="n">
-        <v>120.25</v>
+        <v>255</v>
       </c>
       <c r="D33" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Butter</t>
+          <t>Parathas</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>20.24333333333334</v>
+        <v>14.8575</v>
       </c>
       <c r="C34" t="n">
-        <v>412.1666666666667</v>
+        <v>339.5</v>
       </c>
       <c r="D34" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mops and Brooms</t>
+          <t>Instant Drinks</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>20.03333333333333</v>
+        <v>12.63</v>
       </c>
       <c r="C35" t="n">
-        <v>1023</v>
+        <v>539</v>
       </c>
       <c r="D35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tissues and Napkins</t>
+          <t>Cereals</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>19.95153846153846</v>
+        <v>11.07666666666667</v>
       </c>
       <c r="C36" t="n">
-        <v>118.2307692307692</v>
+        <v>184</v>
       </c>
       <c r="D36" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Frozen Mixed Fruits and Vegetables</t>
+          <t>Disinfectants</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>19.56666666666667</v>
+        <v>10.292</v>
       </c>
       <c r="C37" t="n">
-        <v>336.6666666666667</v>
+        <v>242.8</v>
       </c>
       <c r="D37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Pickles and Olives</t>
+          <t>Tissues and Napkins</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>19.427</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C38" t="n">
-        <v>352.4</v>
+        <v>40</v>
       </c>
       <c r="D38" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Baby Milk</t>
+          <t>packaged-food</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>19.13</v>
+        <v>9.163333333333334</v>
       </c>
       <c r="C39" t="n">
-        <v>255</v>
+        <v>415</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Parathas</t>
+          <t>Traditional Mixes</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>19.08</v>
+        <v>8.172499999999999</v>
       </c>
       <c r="C40" t="n">
-        <v>309.7142857142857</v>
+        <v>32.75</v>
       </c>
       <c r="D40" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kebab and Koftas</t>
+          <t>Cake Mixes and Baking Add Ons</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>18.409</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="C41" t="n">
-        <v>308</v>
+        <v>82</v>
       </c>
       <c r="D41" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Canned Vegetables</t>
+          <t>Butter</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>18.064</v>
+        <v>7.45</v>
       </c>
       <c r="C42" t="n">
-        <v>129.6</v>
+        <v>161.5</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>Cheese</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>17.91333333333333</v>
+        <v>7.325</v>
       </c>
       <c r="C43" t="n">
-        <v>31.66666666666667</v>
+        <v>104.5</v>
       </c>
       <c r="D43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Red Syrups</t>
+          <t>frozen-food</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>16.415</v>
+        <v>7.22</v>
       </c>
       <c r="C44" t="n">
-        <v>363.5</v>
+        <v>155</v>
       </c>
       <c r="D44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jams, Honey and Spreads</t>
+          <t>daily-essentials</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>16.350625</v>
+        <v>6.765</v>
       </c>
       <c r="C45" t="n">
-        <v>326.90625</v>
+        <v>22.5</v>
       </c>
       <c r="D45" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Towels</t>
+          <t>baby-care</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>16.11</v>
+        <v>5</v>
       </c>
       <c r="C46" t="n">
-        <v>110</v>
+        <v>180</v>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Jellies and Custards</t>
+          <t>staples</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>15.18142857142857</v>
+        <v>4.733333333333333</v>
       </c>
       <c r="C47" t="n">
-        <v>46.07142857142857</v>
+        <v>28.33333333333333</v>
       </c>
       <c r="D47" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Cake Mixes and Baking Add Ons</t>
+          <t>Shoe Polish</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>15.16705882352941</v>
+        <v>3.196666666666667</v>
       </c>
       <c r="C48" t="n">
-        <v>247.9411764705882</v>
+        <v>24</v>
       </c>
       <c r="D48" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Cereals</t>
+          <t>Samosas and Rolls</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>14.510625</v>
+        <v>2.33</v>
       </c>
       <c r="C49" t="n">
-        <v>282.3125</v>
+        <v>41</v>
       </c>
       <c r="D49" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -1213,380 +1225,60 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>12.53714285714286</v>
+        <v>2.2</v>
       </c>
       <c r="C50" t="n">
-        <v>386.5714285714286</v>
+        <v>51</v>
       </c>
       <c r="D50" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Instant Drinks</t>
+          <t>Canned Vegetables</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>12.399</v>
+        <v>1.54</v>
       </c>
       <c r="C51" t="n">
-        <v>110.4</v>
+        <v>19</v>
       </c>
       <c r="D51" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Fabric Care</t>
+          <t>Pickles and Olives</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>12.05</v>
+        <v>1.14</v>
       </c>
       <c r="C52" t="n">
-        <v>176.1428571428571</v>
+        <v>6</v>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Insecticides</t>
+          <t>Frozen Seafood</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>11.95</v>
+        <v>0</v>
       </c>
       <c r="C53" t="n">
-        <v>174.1333333333333</v>
+        <v>0</v>
       </c>
       <c r="D53" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Sugar</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>11.53</v>
-      </c>
-      <c r="C54" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="D54" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Shoe Polish</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>11.37416666666667</v>
-      </c>
-      <c r="C55" t="n">
-        <v>61.25</v>
-      </c>
-      <c r="D55" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Samosas and Rolls</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>11.36230769230769</v>
-      </c>
-      <c r="C56" t="n">
-        <v>185</v>
-      </c>
-      <c r="D56" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Plain Yogurt and Flavored yogurt</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>9.813333333333333</v>
-      </c>
-      <c r="C57" t="n">
-        <v>25.66666666666667</v>
-      </c>
-      <c r="D57" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Breads</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>9.58</v>
-      </c>
-      <c r="C58" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="D58" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Frozen Fries</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>7.82</v>
-      </c>
-      <c r="C59" t="n">
-        <v>146</v>
-      </c>
-      <c r="D59" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>frozen-food</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>7.776666666666666</v>
-      </c>
-      <c r="C60" t="n">
-        <v>155</v>
-      </c>
-      <c r="D60" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Traditional Mixes</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>7.075625</v>
-      </c>
-      <c r="C61" t="n">
-        <v>24.9375</v>
-      </c>
-      <c r="D61" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Frozen Seafood</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>6.685</v>
-      </c>
-      <c r="C62" t="n">
-        <v>195</v>
-      </c>
-      <c r="D62" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Margarine</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>6.459000000000001</v>
-      </c>
-      <c r="C63" t="n">
-        <v>95.90000000000001</v>
-      </c>
-      <c r="D63" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>tea-coffee</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>6.390000000000001</v>
-      </c>
-      <c r="C64" t="n">
-        <v>314.3333333333333</v>
-      </c>
-      <c r="D64" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Frozen Meat</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>5.73</v>
-      </c>
-      <c r="C65" t="n">
-        <v>94.25</v>
-      </c>
-      <c r="D65" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Cream</t>
-        </is>
-      </c>
-      <c r="B66" t="n">
-        <v>5.296666666666667</v>
-      </c>
-      <c r="C66" t="n">
-        <v>36.66666666666666</v>
-      </c>
-      <c r="D66" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>meat-poultry</t>
-        </is>
-      </c>
-      <c r="B67" t="n">
-        <v>4.74</v>
-      </c>
-      <c r="C67" t="n">
-        <v>15</v>
-      </c>
-      <c r="D67" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Fresh Fruits</t>
-        </is>
-      </c>
-      <c r="B68" t="n">
-        <v>4.57</v>
-      </c>
-      <c r="C68" t="n">
-        <v>41</v>
-      </c>
-      <c r="D68" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>beverages</t>
-        </is>
-      </c>
-      <c r="B69" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="C69" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D69" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>snacks-beverages</t>
-        </is>
-      </c>
-      <c r="B70" t="n">
-        <v>3.48</v>
-      </c>
-      <c r="C70" t="n">
-        <v>20</v>
-      </c>
-      <c r="D70" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>packaged-food</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
-        <v>1.605</v>
-      </c>
-      <c r="C71" t="n">
-        <v>5</v>
-      </c>
-      <c r="D71" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>daily-essentials</t>
-        </is>
-      </c>
-      <c r="B72" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="C72" t="n">
-        <v>25</v>
-      </c>
-      <c r="D72" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>cooking-oil-ghee</t>
-        </is>
-      </c>
-      <c r="B73" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C73" t="n">
-        <v>4</v>
-      </c>
-      <c r="D73" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: boost matching to 10k+ rows (998 groups, 10002 matched rows)
</commit_message>
<xml_diff>
--- a/analysis/results/category_dispersion.xlsx
+++ b/analysis/results/category_dispersion.xlsx
@@ -453,33 +453,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>chocolates</t>
+          <t>Tea</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>71.15666666666665</v>
+        <v>66.94800000000001</v>
       </c>
       <c r="C2" t="n">
-        <v>679.6666666666666</v>
+        <v>1074.8</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tea</t>
+          <t>chocolates</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66.94800000000001</v>
+        <v>63.31857142857142</v>
       </c>
       <c r="C3" t="n">
-        <v>1074.8</v>
+        <v>2442.714285714286</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -517,17 +517,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>meat-poultry</t>
+          <t>cooking-oil-ghee</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57.12</v>
+        <v>58.29499999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>3113.090909090909</v>
+        <v>5057.5</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -549,14 +549,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pet-care</t>
+          <t>meat-poultry</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52.56</v>
+        <v>53.62846153846154</v>
       </c>
       <c r="C8" t="n">
-        <v>3338.076923076923</v>
+        <v>2746.076923076923</v>
       </c>
       <c r="D8" t="n">
         <v>13</v>
@@ -565,17 +565,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cooking-oil-ghee</t>
+          <t>pet-care</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>49.054</v>
+        <v>52.56</v>
       </c>
       <c r="C9" t="n">
-        <v>4365</v>
+        <v>3338.076923076923</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -597,49 +597,49 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>beverages</t>
+          <t>snacks-beverages</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>45.53599999999999</v>
+        <v>43.12111111111111</v>
       </c>
       <c r="C11" t="n">
-        <v>1319.933333333333</v>
+        <v>388.7777777777778</v>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>snacks-beverages</t>
+          <t>Toilet Supplies</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>43.12111111111111</v>
+        <v>42.51333333333334</v>
       </c>
       <c r="C12" t="n">
-        <v>388.7777777777778</v>
+        <v>730.6666666666666</v>
       </c>
       <c r="D12" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Toilet Supplies</t>
+          <t>beverages</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>42.51333333333334</v>
+        <v>42.13705882352942</v>
       </c>
       <c r="C13" t="n">
-        <v>730.6666666666666</v>
+        <v>1219.294117647059</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14">
@@ -665,13 +665,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.51846153846154</v>
+        <v>40.65642857142858</v>
       </c>
       <c r="C15" t="n">
-        <v>1123.615384615385</v>
+        <v>1125.857142857143</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -693,46 +693,46 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dairy-bakery</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>35.27</v>
+        <v>36.34007220216607</v>
       </c>
       <c r="C17" t="n">
-        <v>200</v>
+        <v>990.1062635379061</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>554</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cakes and Chocolates</t>
+          <t>fruits-vegetables</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>33.70666666666667</v>
+        <v>34.75545454545455</v>
       </c>
       <c r="C18" t="n">
-        <v>79.66666666666667</v>
+        <v>982.8545454545455</v>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>household</t>
+          <t>Cakes and Chocolates</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>33.24</v>
+        <v>33.70666666666667</v>
       </c>
       <c r="C19" t="n">
-        <v>354.6666666666667</v>
+        <v>79.66666666666667</v>
       </c>
       <c r="D19" t="n">
         <v>3</v>
@@ -741,78 +741,78 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>personal-care</t>
+          <t>household</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>30.828</v>
+        <v>33.24</v>
       </c>
       <c r="C20" t="n">
-        <v>534.6</v>
+        <v>354.6666666666667</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Red Syrups</t>
+          <t>personal-care</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>30.18</v>
+        <v>30.865</v>
       </c>
       <c r="C21" t="n">
-        <v>659</v>
+        <v>554.5</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Products</t>
+          <t>Red Syrups</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>28.86702508960573</v>
+        <v>30.18</v>
       </c>
       <c r="C22" t="n">
-        <v>978.9995698924731</v>
+        <v>659</v>
       </c>
       <c r="D22" t="n">
-        <v>279</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>fruits-vegetables</t>
+          <t>dairy-bakery</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>28.715</v>
+        <v>28.5</v>
       </c>
       <c r="C23" t="n">
-        <v>615</v>
+        <v>211</v>
       </c>
       <c r="D23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Detergents and Laundry Soaps</t>
+          <t>baby-care</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>27.5125</v>
+        <v>28.215</v>
       </c>
       <c r="C24" t="n">
-        <v>188.25</v>
+        <v>3241.25</v>
       </c>
       <c r="D24" t="n">
         <v>4</v>
@@ -821,286 +821,286 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Jams, Honey and Spreads</t>
+          <t>Detergents and Laundry Soaps</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>26.71</v>
+        <v>27.5125</v>
       </c>
       <c r="C25" t="n">
-        <v>1499</v>
+        <v>188.25</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Insecticides</t>
+          <t>Jams, Honey and Spreads</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>25.97666666666667</v>
+        <v>26.71</v>
       </c>
       <c r="C26" t="n">
-        <v>472.3333333333333</v>
+        <v>1499</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>tea-coffee</t>
+          <t>Insecticides</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>25.4</v>
+        <v>25.97666666666667</v>
       </c>
       <c r="C27" t="n">
-        <v>1208.416666666667</v>
+        <v>472.3333333333333</v>
       </c>
       <c r="D27" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jellies and Custards</t>
+          <t>tea-coffee</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>23.6425</v>
+        <v>25.4</v>
       </c>
       <c r="C28" t="n">
-        <v>66</v>
+        <v>1208.416666666667</v>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>general</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>22.47307692307692</v>
+        <v>24.64669642857143</v>
       </c>
       <c r="C29" t="n">
-        <v>100.4615384615385</v>
+        <v>1310.814955357143</v>
       </c>
       <c r="D29" t="n">
-        <v>13</v>
+        <v>224</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Noodles and Pasta</t>
+          <t>Jellies and Custards</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>22.194</v>
+        <v>23.6425</v>
       </c>
       <c r="C30" t="n">
-        <v>95.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>snacks</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>21.99582524271845</v>
+        <v>22.47307692307692</v>
       </c>
       <c r="C31" t="n">
-        <v>541.8955339805825</v>
+        <v>100.4615384615385</v>
       </c>
       <c r="D31" t="n">
-        <v>206</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kebab and Koftas</t>
+          <t>Noodles and Pasta</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>19.815</v>
+        <v>22.194</v>
       </c>
       <c r="C32" t="n">
-        <v>406.5</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Baby Milk</t>
+          <t>Kebab and Koftas</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>19.13</v>
+        <v>19.815</v>
       </c>
       <c r="C33" t="n">
-        <v>255</v>
+        <v>406.5</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Parathas</t>
+          <t>Baby Milk</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>14.8575</v>
+        <v>19.13</v>
       </c>
       <c r="C34" t="n">
-        <v>339.5</v>
+        <v>255</v>
       </c>
       <c r="D34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Instant Drinks</t>
+          <t>Parathas</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>12.63</v>
+        <v>14.8575</v>
       </c>
       <c r="C35" t="n">
-        <v>539</v>
+        <v>339.5</v>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cereals</t>
+          <t>Instant Drinks</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>11.07666666666667</v>
+        <v>12.63</v>
       </c>
       <c r="C36" t="n">
-        <v>184</v>
+        <v>539</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Disinfectants</t>
+          <t>Cereals</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>10.292</v>
+        <v>11.07666666666667</v>
       </c>
       <c r="C37" t="n">
-        <v>242.8</v>
+        <v>184</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Tissues and Napkins</t>
+          <t>Disinfectants</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>9.300000000000001</v>
+        <v>10.292</v>
       </c>
       <c r="C38" t="n">
-        <v>40</v>
+        <v>242.8</v>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>packaged-food</t>
+          <t>Tissues and Napkins</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>9.163333333333334</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C39" t="n">
-        <v>415</v>
+        <v>40</v>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Traditional Mixes</t>
+          <t>packaged-food</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>8.172499999999999</v>
+        <v>9.163333333333334</v>
       </c>
       <c r="C40" t="n">
-        <v>32.75</v>
+        <v>415</v>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cake Mixes and Baking Add Ons</t>
+          <t>Traditional Mixes</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>8.029999999999999</v>
+        <v>8.172499999999999</v>
       </c>
       <c r="C41" t="n">
-        <v>82</v>
+        <v>32.75</v>
       </c>
       <c r="D41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Butter</t>
+          <t>Cake Mixes and Baking Add Ons</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>7.45</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="C42" t="n">
-        <v>161.5</v>
+        <v>82</v>
       </c>
       <c r="D42" t="n">
         <v>2</v>
@@ -1109,14 +1109,14 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Cheese</t>
+          <t>Butter</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>7.325</v>
+        <v>7.45</v>
       </c>
       <c r="C43" t="n">
-        <v>104.5</v>
+        <v>161.5</v>
       </c>
       <c r="D43" t="n">
         <v>2</v>
@@ -1125,46 +1125,46 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>frozen-food</t>
+          <t>Cheese</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>7.22</v>
+        <v>7.325</v>
       </c>
       <c r="C44" t="n">
-        <v>155</v>
+        <v>104.5</v>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>daily-essentials</t>
+          <t>frozen-food</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>6.765</v>
+        <v>7.22</v>
       </c>
       <c r="C45" t="n">
-        <v>22.5</v>
+        <v>155</v>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>baby-care</t>
+          <t>daily-essentials</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>5</v>
+        <v>6.765</v>
       </c>
       <c r="C46" t="n">
-        <v>180</v>
+        <v>22.5</v>
       </c>
       <c r="D46" t="n">
         <v>2</v>
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4.733333333333333</v>
+        <v>5.10375</v>
       </c>
       <c r="C47" t="n">
-        <v>28.33333333333333</v>
+        <v>49.125</v>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48">

</xml_diff>